<commit_message>
Obriga preenchimento dos nomes dos acompanhantes
</commit_message>
<xml_diff>
--- a/ANIVERSARIO 60 ANOS.xlsx
+++ b/ANIVERSARIO 60 ANOS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fabrycio\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos\Festa Dona Maria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9143C48F-0B36-4EE5-80B9-EE1E2E0020F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE61388-820D-433E-9B34-F2FA79177D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -733,7 +733,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -761,12 +761,72 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -775,69 +835,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1176,30 +1173,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="E1" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="F1" s="32" t="s">
+      <c r="F1" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="G1" s="36" t="s">
+      <c r="G1" s="22" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="33" t="s">
         <v>129</v>
       </c>
       <c r="B2" s="8" t="s">
@@ -1208,16 +1205,16 @@
       <c r="C2" s="4">
         <v>1</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="E2" s="33">
+      <c r="E2" s="25">
         <v>18</v>
       </c>
-      <c r="F2" s="34" t="s">
+      <c r="F2" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="33" t="s">
+      <c r="G2" s="25" t="s">
         <v>157</v>
       </c>
       <c r="R2" s="1"/>
@@ -1227,19 +1224,19 @@
       <c r="W2" s="1"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A3" s="14"/>
+      <c r="A3" s="34"/>
       <c r="B3" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C3" s="4">
         <v>2</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="33"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="33"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="25"/>
       <c r="R3" s="1"/>
       <c r="S3" s="3"/>
       <c r="T3" s="1"/>
@@ -1247,19 +1244,19 @@
       <c r="W3" s="1"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A4" s="14"/>
+      <c r="A4" s="34"/>
       <c r="B4" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C4" s="4">
         <v>3</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="33"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="33"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="25"/>
       <c r="R4" s="1"/>
       <c r="S4" s="3"/>
       <c r="T4" s="1"/>
@@ -1267,19 +1264,19 @@
       <c r="W4" s="1"/>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A5" s="14"/>
+      <c r="A5" s="34"/>
       <c r="B5" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C5" s="4">
         <v>4</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="33"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="33"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="25"/>
       <c r="R5" s="1"/>
       <c r="S5" s="3"/>
       <c r="T5" s="1"/>
@@ -1287,19 +1284,19 @@
       <c r="W5" s="1"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A6" s="14"/>
+      <c r="A6" s="34"/>
       <c r="B6" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C6" s="4">
         <v>5</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="33"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="33"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="25"/>
       <c r="R6" s="1"/>
       <c r="S6" s="3"/>
       <c r="T6" s="1"/>
@@ -1307,19 +1304,19 @@
       <c r="W6" s="1"/>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A7" s="14"/>
+      <c r="A7" s="34"/>
       <c r="B7" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C7" s="4">
         <v>6</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="33"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="25"/>
       <c r="R7" s="1"/>
       <c r="S7" s="3"/>
       <c r="T7" s="1"/>
@@ -1327,19 +1324,19 @@
       <c r="W7" s="1"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A8" s="14"/>
+      <c r="A8" s="34"/>
       <c r="B8" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C8" s="4">
         <v>7</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="33"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="25"/>
       <c r="R8" s="1"/>
       <c r="S8" s="3"/>
       <c r="T8" s="1"/>
@@ -1347,19 +1344,19 @@
       <c r="W8" s="1"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A9" s="14"/>
+      <c r="A9" s="34"/>
       <c r="B9" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C9" s="4">
         <v>8</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="33"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="25"/>
       <c r="R9" s="1"/>
       <c r="S9" s="3"/>
       <c r="T9" s="1"/>
@@ -1367,19 +1364,19 @@
       <c r="W9" s="1"/>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A10" s="14"/>
+      <c r="A10" s="34"/>
       <c r="B10" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C10" s="4">
         <v>9</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="33"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="33"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="25"/>
       <c r="R10" s="1"/>
       <c r="S10" s="3"/>
       <c r="T10" s="1"/>
@@ -1387,19 +1384,19 @@
       <c r="W10" s="1"/>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A11" s="14"/>
+      <c r="A11" s="34"/>
       <c r="B11" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C11" s="4">
         <v>10</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="33"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="33"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="25"/>
       <c r="R11" s="1"/>
       <c r="S11" s="3"/>
       <c r="T11" s="1"/>
@@ -1407,19 +1404,19 @@
       <c r="W11" s="1"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A12" s="14"/>
+      <c r="A12" s="34"/>
       <c r="B12" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C12" s="4">
         <v>11</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="33"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="33"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="25"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
@@ -1427,43 +1424,43 @@
       <c r="W12" s="1"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A13" s="14"/>
+      <c r="A13" s="34"/>
       <c r="B13" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C13" s="4">
         <v>12</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="33"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="33"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="25"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A14" s="14"/>
+      <c r="A14" s="34"/>
       <c r="B14" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C14" s="4">
         <v>13</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="33"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="33"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="25"/>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A15" s="14"/>
+      <c r="A15" s="34"/>
       <c r="B15" s="7" t="s">
         <v>0</v>
       </c>
@@ -1473,15 +1470,15 @@
       <c r="D15" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="33"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="33"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="25"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A16" s="14"/>
+      <c r="A16" s="34"/>
       <c r="B16" s="7" t="s">
         <v>0</v>
       </c>
@@ -1491,15 +1488,15 @@
       <c r="D16" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="33"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="33"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="25"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A17" s="14"/>
+      <c r="A17" s="34"/>
       <c r="B17" s="7" t="s">
         <v>0</v>
       </c>
@@ -1509,15 +1506,15 @@
       <c r="D17" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="33"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="33"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="25"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A18" s="14"/>
+      <c r="A18" s="34"/>
       <c r="B18" s="7" t="s">
         <v>0</v>
       </c>
@@ -1527,15 +1524,15 @@
       <c r="D18" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E18" s="33"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="33"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="25"/>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
       <c r="T18" s="1"/>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A19" s="15"/>
+      <c r="A19" s="35"/>
       <c r="B19" s="7" t="s">
         <v>0</v>
       </c>
@@ -1545,15 +1542,15 @@
       <c r="D19" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="33"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="33"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="25"/>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="32" t="s">
         <v>98</v>
       </c>
       <c r="B20" s="8" t="s">
@@ -1562,16 +1559,16 @@
       <c r="C20" s="4">
         <v>19</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="E20" s="33">
+      <c r="E20" s="25">
         <v>3</v>
       </c>
-      <c r="F20" s="34" t="s">
+      <c r="F20" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="G20" s="33"/>
+      <c r="G20" s="25"/>
       <c r="N20" s="5"/>
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
@@ -1580,26 +1577,26 @@
       <c r="W20" s="1"/>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A21" s="19"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C21" s="4">
         <v>20</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="D21" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="33"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="25"/>
       <c r="N21" s="5"/>
       <c r="S21" s="1"/>
       <c r="U21" s="1"/>
       <c r="W21" s="1"/>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A22" s="19"/>
+      <c r="A22" s="32"/>
       <c r="B22" s="7" t="s">
         <v>0</v>
       </c>
@@ -1609,16 +1606,16 @@
       <c r="D22" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="E22" s="33"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="33"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="25"/>
       <c r="N22" s="5"/>
       <c r="S22" s="1"/>
       <c r="U22" s="1"/>
       <c r="W22" s="1"/>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="29" t="s">
         <v>99</v>
       </c>
       <c r="B23" s="8" t="s">
@@ -1627,76 +1624,76 @@
       <c r="C23" s="4">
         <v>22</v>
       </c>
-      <c r="D23" s="22" t="s">
+      <c r="D23" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="E23" s="33">
+      <c r="E23" s="25">
         <v>5</v>
       </c>
-      <c r="F23" s="34" t="s">
+      <c r="F23" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="G23" s="33"/>
+      <c r="G23" s="25"/>
       <c r="N23" s="5"/>
       <c r="S23" s="1"/>
       <c r="U23" s="1"/>
       <c r="W23" s="1"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A24" s="12"/>
+      <c r="A24" s="30"/>
       <c r="B24" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C24" s="4">
         <v>23</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="D24" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="E24" s="33"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="33"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="25"/>
       <c r="N24" s="5"/>
       <c r="S24" s="1"/>
       <c r="U24" s="1"/>
       <c r="W24" s="1"/>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A25" s="12"/>
+      <c r="A25" s="30"/>
       <c r="B25" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C25" s="4">
         <v>24</v>
       </c>
-      <c r="D25" s="22" t="s">
+      <c r="D25" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="33"/>
-      <c r="F25" s="30"/>
-      <c r="G25" s="33"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="25"/>
       <c r="S25" s="1"/>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A26" s="12"/>
+      <c r="A26" s="30"/>
       <c r="B26" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C26" s="4">
         <v>25</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="D26" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E26" s="33"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="33"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="25"/>
       <c r="S26" s="1"/>
       <c r="U26" s="1"/>
       <c r="W26" s="1"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A27" s="16"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="7" t="s">
         <v>0</v>
       </c>
@@ -1706,15 +1703,15 @@
       <c r="D27" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E27" s="33"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="33"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="25"/>
       <c r="S27" s="1"/>
       <c r="U27" s="1"/>
       <c r="W27" s="1"/>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="32" t="s">
         <v>100</v>
       </c>
       <c r="B28" s="8" t="s">
@@ -1723,70 +1720,70 @@
       <c r="C28" s="4">
         <v>27</v>
       </c>
-      <c r="D28" s="23" t="s">
+      <c r="D28" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="E28" s="33">
+      <c r="E28" s="25">
         <v>4</v>
       </c>
-      <c r="F28" s="34" t="s">
+      <c r="F28" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="G28" s="33"/>
+      <c r="G28" s="25"/>
       <c r="U28" s="1"/>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A29" s="19"/>
+      <c r="A29" s="32"/>
       <c r="B29" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C29" s="4">
         <v>28</v>
       </c>
-      <c r="D29" s="23" t="s">
+      <c r="D29" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="33"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="25"/>
       <c r="S29" s="1"/>
       <c r="U29" s="1"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A30" s="18"/>
+      <c r="A30" s="28"/>
       <c r="B30" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C30" s="4">
         <v>29</v>
       </c>
-      <c r="D30" s="23" t="s">
+      <c r="D30" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="E30" s="33"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="33"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="25"/>
       <c r="S30" s="1"/>
       <c r="U30" s="1"/>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A31" s="18"/>
+      <c r="A31" s="28"/>
       <c r="B31" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C31" s="4">
         <v>30</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="D31" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="33"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="33"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="25"/>
       <c r="U31" s="1"/>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.4">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="11" t="s">
         <v>101</v>
       </c>
       <c r="B32" s="8" t="s">
@@ -1795,20 +1792,20 @@
       <c r="C32" s="4">
         <v>31</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="D32" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="E32" s="32">
+      <c r="E32" s="23">
         <v>1</v>
       </c>
-      <c r="F32" s="35" t="s">
+      <c r="F32" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="G32" s="32"/>
+      <c r="G32" s="23"/>
       <c r="U32" s="1"/>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="29" t="s">
         <v>102</v>
       </c>
       <c r="B33" s="8" t="s">
@@ -1817,88 +1814,88 @@
       <c r="C33" s="4">
         <v>32</v>
       </c>
-      <c r="D33" s="24" t="s">
+      <c r="D33" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="E33" s="33">
+      <c r="E33" s="25">
         <v>6</v>
       </c>
-      <c r="F33" s="34" t="s">
+      <c r="F33" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="G33" s="33"/>
+      <c r="G33" s="25"/>
       <c r="U33" s="1"/>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A34" s="12"/>
+      <c r="A34" s="30"/>
       <c r="B34" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C34" s="4">
         <v>33</v>
       </c>
-      <c r="D34" s="24" t="s">
+      <c r="D34" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="E34" s="33"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="33"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="25"/>
       <c r="S34" s="1"/>
       <c r="U34" s="1"/>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A35" s="12"/>
+      <c r="A35" s="30"/>
       <c r="B35" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C35" s="4">
         <v>34</v>
       </c>
-      <c r="D35" s="24" t="s">
+      <c r="D35" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E35" s="33"/>
-      <c r="F35" s="30"/>
-      <c r="G35" s="33"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="25"/>
       <c r="S35" s="1"/>
       <c r="U35" s="1"/>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A36" s="12"/>
+      <c r="A36" s="30"/>
       <c r="B36" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C36" s="4">
         <v>35</v>
       </c>
-      <c r="D36" s="24" t="s">
+      <c r="D36" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="E36" s="33"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="33"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="25"/>
       <c r="S36" s="1"/>
       <c r="U36" s="1"/>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A37" s="12"/>
+      <c r="A37" s="30"/>
       <c r="B37" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C37" s="4">
         <v>36</v>
       </c>
-      <c r="D37" s="24" t="s">
+      <c r="D37" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="E37" s="33"/>
-      <c r="F37" s="30"/>
-      <c r="G37" s="33"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="25"/>
       <c r="S37" s="1"/>
       <c r="U37" s="1"/>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A38" s="16"/>
+      <c r="A38" s="31"/>
       <c r="B38" s="7" t="s">
         <v>0</v>
       </c>
@@ -1908,14 +1905,14 @@
       <c r="D38" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="33"/>
-      <c r="F38" s="30"/>
-      <c r="G38" s="33"/>
+      <c r="E38" s="25"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="25"/>
       <c r="S38" s="1"/>
       <c r="U38" s="1"/>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A39" s="11" t="s">
+      <c r="A39" s="29" t="s">
         <v>103</v>
       </c>
       <c r="B39" s="8" t="s">
@@ -1924,69 +1921,69 @@
       <c r="C39" s="4">
         <v>38</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D39" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E39" s="33">
+      <c r="E39" s="25">
         <v>5</v>
       </c>
-      <c r="F39" s="34" t="s">
+      <c r="F39" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="G39" s="33"/>
+      <c r="G39" s="25"/>
       <c r="S39" s="1"/>
       <c r="U39" s="1"/>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A40" s="12"/>
+      <c r="A40" s="30"/>
       <c r="B40" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C40" s="4">
         <v>39</v>
       </c>
-      <c r="D40" s="20" t="s">
+      <c r="D40" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="E40" s="33"/>
-      <c r="F40" s="30"/>
-      <c r="G40" s="33"/>
+      <c r="E40" s="25"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="25"/>
       <c r="S40" s="1"/>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A41" s="12"/>
+      <c r="A41" s="30"/>
       <c r="B41" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C41" s="4">
         <v>40</v>
       </c>
-      <c r="D41" s="20" t="s">
+      <c r="D41" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="E41" s="33"/>
-      <c r="F41" s="30"/>
-      <c r="G41" s="33"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="25"/>
       <c r="S41" s="1"/>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A42" s="12"/>
+      <c r="A42" s="30"/>
       <c r="B42" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C42" s="4">
         <v>41</v>
       </c>
-      <c r="D42" s="20" t="s">
+      <c r="D42" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="E42" s="33"/>
-      <c r="F42" s="30"/>
-      <c r="G42" s="33"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="27"/>
+      <c r="G42" s="25"/>
       <c r="S42" s="1"/>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A43" s="16"/>
+      <c r="A43" s="31"/>
       <c r="B43" s="7" t="s">
         <v>0</v>
       </c>
@@ -1996,13 +1993,13 @@
       <c r="D43" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E43" s="33"/>
-      <c r="F43" s="30"/>
-      <c r="G43" s="33"/>
+      <c r="E43" s="25"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="25"/>
       <c r="S43" s="1"/>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A44" s="19" t="s">
+      <c r="A44" s="32" t="s">
         <v>104</v>
       </c>
       <c r="B44" s="8" t="s">
@@ -2011,67 +2008,67 @@
       <c r="C44" s="4">
         <v>43</v>
       </c>
-      <c r="D44" s="21" t="s">
+      <c r="D44" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="E44" s="33">
+      <c r="E44" s="25">
         <v>4</v>
       </c>
-      <c r="F44" s="34" t="s">
+      <c r="F44" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="G44" s="33"/>
+      <c r="G44" s="25"/>
       <c r="S44" s="1"/>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A45" s="19"/>
+      <c r="A45" s="32"/>
       <c r="B45" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C45" s="4">
         <v>44</v>
       </c>
-      <c r="D45" s="21" t="s">
+      <c r="D45" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E45" s="33"/>
-      <c r="F45" s="30"/>
-      <c r="G45" s="33"/>
+      <c r="E45" s="25"/>
+      <c r="F45" s="27"/>
+      <c r="G45" s="25"/>
       <c r="S45" s="1"/>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A46" s="18"/>
+      <c r="A46" s="28"/>
       <c r="B46" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C46" s="4">
         <v>45</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="D46" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="E46" s="33"/>
-      <c r="F46" s="30"/>
-      <c r="G46" s="33"/>
+      <c r="E46" s="25"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="25"/>
       <c r="S46" s="1"/>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A47" s="18"/>
+      <c r="A47" s="28"/>
       <c r="B47" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C47" s="4">
         <v>46</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="D47" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E47" s="33"/>
-      <c r="F47" s="30"/>
-      <c r="G47" s="33"/>
+      <c r="E47" s="25"/>
+      <c r="F47" s="27"/>
+      <c r="G47" s="25"/>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A48" s="17" t="s">
+      <c r="A48" s="11" t="s">
         <v>106</v>
       </c>
       <c r="B48" s="8" t="s">
@@ -2080,19 +2077,19 @@
       <c r="C48" s="4">
         <v>47</v>
       </c>
-      <c r="D48" s="21" t="s">
+      <c r="D48" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E48" s="32">
+      <c r="E48" s="23">
         <v>1</v>
       </c>
-      <c r="F48" s="35" t="s">
+      <c r="F48" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="G48" s="32"/>
+      <c r="G48" s="23"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A49" s="18" t="s">
+      <c r="A49" s="28" t="s">
         <v>108</v>
       </c>
       <c r="B49" s="8" t="s">
@@ -2101,34 +2098,34 @@
       <c r="C49" s="4">
         <v>48</v>
       </c>
-      <c r="D49" s="25" t="s">
+      <c r="D49" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="E49" s="33">
+      <c r="E49" s="25">
         <v>2</v>
       </c>
-      <c r="F49" s="34" t="s">
+      <c r="F49" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="G49" s="33"/>
+      <c r="G49" s="25"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A50" s="18"/>
+      <c r="A50" s="28"/>
       <c r="B50" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C50" s="4">
         <v>49</v>
       </c>
-      <c r="D50" s="25" t="s">
+      <c r="D50" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="E50" s="33"/>
-      <c r="F50" s="30"/>
-      <c r="G50" s="33"/>
+      <c r="E50" s="25"/>
+      <c r="F50" s="27"/>
+      <c r="G50" s="25"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A51" s="18" t="s">
+      <c r="A51" s="28" t="s">
         <v>107</v>
       </c>
       <c r="B51" s="8" t="s">
@@ -2137,79 +2134,79 @@
       <c r="C51" s="4">
         <v>50</v>
       </c>
-      <c r="D51" s="26" t="s">
+      <c r="D51" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E51" s="33">
+      <c r="E51" s="25">
         <v>5</v>
       </c>
-      <c r="F51" s="34" t="s">
+      <c r="F51" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="G51" s="33"/>
+      <c r="G51" s="25"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A52" s="18"/>
+      <c r="A52" s="28"/>
       <c r="B52" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C52" s="4">
         <v>51</v>
       </c>
-      <c r="D52" s="26" t="s">
+      <c r="D52" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="E52" s="33"/>
-      <c r="F52" s="30"/>
-      <c r="G52" s="33"/>
+      <c r="E52" s="25"/>
+      <c r="F52" s="27"/>
+      <c r="G52" s="25"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A53" s="18"/>
+      <c r="A53" s="28"/>
       <c r="B53" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C53" s="4">
         <v>52</v>
       </c>
-      <c r="D53" s="26" t="s">
+      <c r="D53" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="E53" s="33"/>
-      <c r="F53" s="30"/>
-      <c r="G53" s="33"/>
+      <c r="E53" s="25"/>
+      <c r="F53" s="27"/>
+      <c r="G53" s="25"/>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A54" s="18"/>
+      <c r="A54" s="28"/>
       <c r="B54" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C54" s="4">
         <v>53</v>
       </c>
-      <c r="D54" s="26" t="s">
+      <c r="D54" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="E54" s="33"/>
-      <c r="F54" s="30"/>
-      <c r="G54" s="33"/>
+      <c r="E54" s="25"/>
+      <c r="F54" s="27"/>
+      <c r="G54" s="25"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A55" s="18"/>
+      <c r="A55" s="28"/>
       <c r="B55" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C55" s="4">
         <v>54</v>
       </c>
-      <c r="D55" s="26" t="s">
+      <c r="D55" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="E55" s="33"/>
-      <c r="F55" s="30"/>
-      <c r="G55" s="33"/>
+      <c r="E55" s="25"/>
+      <c r="F55" s="27"/>
+      <c r="G55" s="25"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A56" s="18" t="s">
+      <c r="A56" s="28" t="s">
         <v>109</v>
       </c>
       <c r="B56" s="8" t="s">
@@ -2218,64 +2215,64 @@
       <c r="C56" s="4">
         <v>55</v>
       </c>
-      <c r="D56" s="21" t="s">
+      <c r="D56" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E56" s="33">
+      <c r="E56" s="25">
         <v>4</v>
       </c>
-      <c r="F56" s="34" t="s">
+      <c r="F56" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="G56" s="33"/>
+      <c r="G56" s="25"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A57" s="18"/>
+      <c r="A57" s="28"/>
       <c r="B57" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C57" s="4">
         <v>56</v>
       </c>
-      <c r="D57" s="21" t="s">
+      <c r="D57" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="E57" s="33"/>
-      <c r="F57" s="30"/>
-      <c r="G57" s="33"/>
+      <c r="E57" s="25"/>
+      <c r="F57" s="27"/>
+      <c r="G57" s="25"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A58" s="18"/>
+      <c r="A58" s="28"/>
       <c r="B58" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C58" s="4">
         <v>57</v>
       </c>
-      <c r="D58" s="21" t="s">
+      <c r="D58" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="E58" s="33"/>
-      <c r="F58" s="30"/>
-      <c r="G58" s="33"/>
+      <c r="E58" s="25"/>
+      <c r="F58" s="27"/>
+      <c r="G58" s="25"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A59" s="18"/>
+      <c r="A59" s="28"/>
       <c r="B59" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C59" s="4">
         <v>58</v>
       </c>
-      <c r="D59" s="21" t="s">
+      <c r="D59" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="E59" s="33"/>
-      <c r="F59" s="30"/>
-      <c r="G59" s="33"/>
+      <c r="E59" s="25"/>
+      <c r="F59" s="27"/>
+      <c r="G59" s="25"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A60" s="11" t="s">
+      <c r="A60" s="29" t="s">
         <v>120</v>
       </c>
       <c r="B60" s="8" t="s">
@@ -2284,129 +2281,129 @@
       <c r="C60" s="4">
         <v>59</v>
       </c>
-      <c r="D60" s="27" t="s">
+      <c r="D60" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="E60" s="33">
+      <c r="E60" s="25">
         <v>9</v>
       </c>
-      <c r="F60" s="34" t="s">
+      <c r="F60" s="26" t="s">
         <v>142</v>
       </c>
-      <c r="G60" s="33"/>
+      <c r="G60" s="25"/>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A61" s="12"/>
+      <c r="A61" s="30"/>
       <c r="B61" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C61" s="4">
         <v>60</v>
       </c>
-      <c r="D61" s="27" t="s">
+      <c r="D61" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="E61" s="33"/>
-      <c r="F61" s="30"/>
-      <c r="G61" s="33"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="27"/>
+      <c r="G61" s="25"/>
       <c r="K61" s="1"/>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A62" s="12"/>
+      <c r="A62" s="30"/>
       <c r="B62" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C62" s="4">
         <v>61</v>
       </c>
-      <c r="D62" s="27" t="s">
+      <c r="D62" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="E62" s="33"/>
-      <c r="F62" s="30"/>
-      <c r="G62" s="33"/>
+      <c r="E62" s="25"/>
+      <c r="F62" s="27"/>
+      <c r="G62" s="25"/>
       <c r="K62" s="1"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A63" s="12"/>
+      <c r="A63" s="30"/>
       <c r="B63" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C63" s="4">
         <v>62</v>
       </c>
-      <c r="D63" s="27" t="s">
+      <c r="D63" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E63" s="33"/>
-      <c r="F63" s="30"/>
-      <c r="G63" s="33"/>
+      <c r="E63" s="25"/>
+      <c r="F63" s="27"/>
+      <c r="G63" s="25"/>
       <c r="K63" s="1"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A64" s="12"/>
+      <c r="A64" s="30"/>
       <c r="B64" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C64" s="4">
         <v>63</v>
       </c>
-      <c r="D64" s="27" t="s">
+      <c r="D64" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="E64" s="33"/>
-      <c r="F64" s="30"/>
-      <c r="G64" s="33"/>
+      <c r="E64" s="25"/>
+      <c r="F64" s="27"/>
+      <c r="G64" s="25"/>
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A65" s="12"/>
+      <c r="A65" s="30"/>
       <c r="B65" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C65" s="4">
         <v>64</v>
       </c>
-      <c r="D65" s="27" t="s">
+      <c r="D65" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E65" s="33"/>
-      <c r="F65" s="30"/>
-      <c r="G65" s="33"/>
+      <c r="E65" s="25"/>
+      <c r="F65" s="27"/>
+      <c r="G65" s="25"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A66" s="12"/>
+      <c r="A66" s="30"/>
       <c r="B66" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C66" s="4">
         <v>65</v>
       </c>
-      <c r="D66" s="27" t="s">
+      <c r="D66" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E66" s="33"/>
-      <c r="F66" s="30"/>
-      <c r="G66" s="33"/>
+      <c r="E66" s="25"/>
+      <c r="F66" s="27"/>
+      <c r="G66" s="25"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A67" s="12"/>
+      <c r="A67" s="30"/>
       <c r="B67" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C67" s="4">
         <v>66</v>
       </c>
-      <c r="D67" s="27" t="s">
+      <c r="D67" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="E67" s="33"/>
-      <c r="F67" s="30"/>
-      <c r="G67" s="33"/>
+      <c r="E67" s="25"/>
+      <c r="F67" s="27"/>
+      <c r="G67" s="25"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A68" s="16"/>
+      <c r="A68" s="31"/>
       <c r="B68" s="7" t="s">
         <v>0</v>
       </c>
@@ -2416,12 +2413,12 @@
       <c r="D68" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E68" s="33"/>
-      <c r="F68" s="30"/>
-      <c r="G68" s="33"/>
+      <c r="E68" s="25"/>
+      <c r="F68" s="27"/>
+      <c r="G68" s="25"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A69" s="19" t="s">
+      <c r="A69" s="32" t="s">
         <v>121</v>
       </c>
       <c r="B69" s="8" t="s">
@@ -2430,34 +2427,34 @@
       <c r="C69" s="4">
         <v>68</v>
       </c>
-      <c r="D69" s="20" t="s">
+      <c r="D69" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E69" s="33">
+      <c r="E69" s="25">
         <v>2</v>
       </c>
-      <c r="F69" s="34" t="s">
+      <c r="F69" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="G69" s="33"/>
+      <c r="G69" s="25"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A70" s="18"/>
+      <c r="A70" s="28"/>
       <c r="B70" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C70" s="4">
         <v>69</v>
       </c>
-      <c r="D70" s="20" t="s">
+      <c r="D70" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="E70" s="33"/>
-      <c r="F70" s="30"/>
-      <c r="G70" s="33"/>
+      <c r="E70" s="25"/>
+      <c r="F70" s="27"/>
+      <c r="G70" s="25"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A71" s="18" t="s">
+      <c r="A71" s="28" t="s">
         <v>110</v>
       </c>
       <c r="B71" s="8" t="s">
@@ -2466,49 +2463,49 @@
       <c r="C71" s="4">
         <v>70</v>
       </c>
-      <c r="D71" s="24" t="s">
+      <c r="D71" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="E71" s="33">
+      <c r="E71" s="25">
         <v>3</v>
       </c>
-      <c r="F71" s="34" t="s">
+      <c r="F71" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="G71" s="33"/>
+      <c r="G71" s="25"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A72" s="18"/>
+      <c r="A72" s="28"/>
       <c r="B72" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C72" s="4">
         <v>71</v>
       </c>
-      <c r="D72" s="24" t="s">
+      <c r="D72" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="E72" s="33"/>
-      <c r="F72" s="30"/>
-      <c r="G72" s="33"/>
+      <c r="E72" s="25"/>
+      <c r="F72" s="27"/>
+      <c r="G72" s="25"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A73" s="18"/>
+      <c r="A73" s="28"/>
       <c r="B73" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C73" s="4">
         <v>72</v>
       </c>
-      <c r="D73" s="24" t="s">
+      <c r="D73" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="E73" s="33"/>
-      <c r="F73" s="30"/>
-      <c r="G73" s="33"/>
+      <c r="E73" s="25"/>
+      <c r="F73" s="27"/>
+      <c r="G73" s="25"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A74" s="18" t="s">
+      <c r="A74" s="28" t="s">
         <v>111</v>
       </c>
       <c r="B74" s="8" t="s">
@@ -2517,64 +2514,64 @@
       <c r="C74" s="4">
         <v>73</v>
       </c>
-      <c r="D74" s="20" t="s">
+      <c r="D74" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E74" s="33">
+      <c r="E74" s="25">
         <v>4</v>
       </c>
-      <c r="F74" s="34" t="s">
+      <c r="F74" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="G74" s="33"/>
+      <c r="G74" s="25"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A75" s="18"/>
+      <c r="A75" s="28"/>
       <c r="B75" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C75" s="4">
         <v>74</v>
       </c>
-      <c r="D75" s="20" t="s">
+      <c r="D75" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="E75" s="33"/>
-      <c r="F75" s="30"/>
-      <c r="G75" s="33"/>
+      <c r="E75" s="25"/>
+      <c r="F75" s="27"/>
+      <c r="G75" s="25"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A76" s="18"/>
+      <c r="A76" s="28"/>
       <c r="B76" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C76" s="4">
         <v>75</v>
       </c>
-      <c r="D76" s="20" t="s">
+      <c r="D76" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="E76" s="33"/>
-      <c r="F76" s="30"/>
-      <c r="G76" s="33"/>
+      <c r="E76" s="25"/>
+      <c r="F76" s="27"/>
+      <c r="G76" s="25"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A77" s="18"/>
+      <c r="A77" s="28"/>
       <c r="B77" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C77" s="4">
         <v>76</v>
       </c>
-      <c r="D77" s="20" t="s">
+      <c r="D77" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="E77" s="33"/>
-      <c r="F77" s="30"/>
-      <c r="G77" s="33"/>
+      <c r="E77" s="25"/>
+      <c r="F77" s="27"/>
+      <c r="G77" s="25"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A78" s="17" t="s">
+      <c r="A78" s="11" t="s">
         <v>127</v>
       </c>
       <c r="B78" s="8" t="s">
@@ -2583,19 +2580,19 @@
       <c r="C78" s="4">
         <v>77</v>
       </c>
-      <c r="D78" s="24" t="s">
+      <c r="D78" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="E78" s="32">
+      <c r="E78" s="23">
         <v>1</v>
       </c>
-      <c r="F78" s="35" t="s">
+      <c r="F78" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="G78" s="32"/>
+      <c r="G78" s="23"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A79" s="17" t="s">
+      <c r="A79" s="11" t="s">
         <v>128</v>
       </c>
       <c r="B79" s="8" t="s">
@@ -2604,19 +2601,19 @@
       <c r="C79" s="4">
         <v>78</v>
       </c>
-      <c r="D79" s="21" t="s">
+      <c r="D79" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="E79" s="32">
+      <c r="E79" s="23">
         <v>1</v>
       </c>
-      <c r="F79" s="35" t="s">
+      <c r="F79" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="G79" s="32"/>
+      <c r="G79" s="23"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A80" s="18" t="s">
+      <c r="A80" s="28" t="s">
         <v>112</v>
       </c>
       <c r="B80" s="8" t="s">
@@ -2625,34 +2622,34 @@
       <c r="C80" s="4">
         <v>79</v>
       </c>
-      <c r="D80" s="28" t="s">
+      <c r="D80" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="E80" s="33">
+      <c r="E80" s="25">
         <v>2</v>
       </c>
-      <c r="F80" s="34" t="s">
+      <c r="F80" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="G80" s="33"/>
+      <c r="G80" s="25"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A81" s="18"/>
+      <c r="A81" s="28"/>
       <c r="B81" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C81" s="4">
         <v>80</v>
       </c>
-      <c r="D81" s="28" t="s">
+      <c r="D81" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="E81" s="33"/>
-      <c r="F81" s="30"/>
-      <c r="G81" s="33"/>
+      <c r="E81" s="25"/>
+      <c r="F81" s="27"/>
+      <c r="G81" s="25"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A82" s="18" t="s">
+      <c r="A82" s="28" t="s">
         <v>114</v>
       </c>
       <c r="B82" s="8" t="s">
@@ -2661,34 +2658,34 @@
       <c r="C82" s="4">
         <v>81</v>
       </c>
-      <c r="D82" s="29" t="s">
+      <c r="D82" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="E82" s="33">
+      <c r="E82" s="25">
         <v>2</v>
       </c>
-      <c r="F82" s="34" t="s">
+      <c r="F82" s="26" t="s">
         <v>149</v>
       </c>
-      <c r="G82" s="33"/>
+      <c r="G82" s="25"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A83" s="18"/>
+      <c r="A83" s="28"/>
       <c r="B83" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C83" s="4">
         <v>82</v>
       </c>
-      <c r="D83" s="29" t="s">
+      <c r="D83" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="E83" s="33"/>
-      <c r="F83" s="30"/>
-      <c r="G83" s="33"/>
+      <c r="E83" s="25"/>
+      <c r="F83" s="27"/>
+      <c r="G83" s="25"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A84" s="18" t="s">
+      <c r="A84" s="28" t="s">
         <v>113</v>
       </c>
       <c r="B84" s="8" t="s">
@@ -2697,64 +2694,64 @@
       <c r="C84" s="4">
         <v>83</v>
       </c>
-      <c r="D84" s="20" t="s">
+      <c r="D84" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E84" s="33">
+      <c r="E84" s="25">
         <v>4</v>
       </c>
-      <c r="F84" s="34" t="s">
+      <c r="F84" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="G84" s="33"/>
+      <c r="G84" s="25"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A85" s="18"/>
+      <c r="A85" s="28"/>
       <c r="B85" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C85" s="4">
         <v>84</v>
       </c>
-      <c r="D85" s="20" t="s">
+      <c r="D85" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="E85" s="33"/>
-      <c r="F85" s="30"/>
-      <c r="G85" s="33"/>
+      <c r="E85" s="25"/>
+      <c r="F85" s="27"/>
+      <c r="G85" s="25"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A86" s="18"/>
+      <c r="A86" s="28"/>
       <c r="B86" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C86" s="4">
         <v>85</v>
       </c>
-      <c r="D86" s="20" t="s">
+      <c r="D86" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="E86" s="33"/>
-      <c r="F86" s="30"/>
-      <c r="G86" s="33"/>
+      <c r="E86" s="25"/>
+      <c r="F86" s="27"/>
+      <c r="G86" s="25"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A87" s="18"/>
+      <c r="A87" s="28"/>
       <c r="B87" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C87" s="4">
         <v>86</v>
       </c>
-      <c r="D87" s="20" t="s">
+      <c r="D87" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="E87" s="33"/>
-      <c r="F87" s="30"/>
-      <c r="G87" s="33"/>
+      <c r="E87" s="25"/>
+      <c r="F87" s="27"/>
+      <c r="G87" s="25"/>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A88" s="18" t="s">
+      <c r="A88" s="28" t="s">
         <v>115</v>
       </c>
       <c r="B88" s="8" t="s">
@@ -2763,49 +2760,49 @@
       <c r="C88" s="4">
         <v>87</v>
       </c>
-      <c r="D88" s="24" t="s">
+      <c r="D88" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="E88" s="33">
+      <c r="E88" s="25">
         <v>3</v>
       </c>
-      <c r="F88" s="34" t="s">
+      <c r="F88" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="G88" s="33"/>
+      <c r="G88" s="25"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A89" s="18"/>
+      <c r="A89" s="28"/>
       <c r="B89" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C89" s="4">
         <v>88</v>
       </c>
-      <c r="D89" s="24" t="s">
+      <c r="D89" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="E89" s="33"/>
-      <c r="F89" s="30"/>
-      <c r="G89" s="33"/>
+      <c r="E89" s="25"/>
+      <c r="F89" s="27"/>
+      <c r="G89" s="25"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A90" s="18"/>
+      <c r="A90" s="28"/>
       <c r="B90" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C90" s="4">
         <v>89</v>
       </c>
-      <c r="D90" s="24" t="s">
+      <c r="D90" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="E90" s="33"/>
-      <c r="F90" s="30"/>
-      <c r="G90" s="33"/>
+      <c r="E90" s="25"/>
+      <c r="F90" s="27"/>
+      <c r="G90" s="25"/>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A91" s="18" t="s">
+      <c r="A91" s="28" t="s">
         <v>116</v>
       </c>
       <c r="B91" s="8" t="s">
@@ -2814,64 +2811,64 @@
       <c r="C91" s="4">
         <v>90</v>
       </c>
-      <c r="D91" s="21" t="s">
+      <c r="D91" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="E91" s="33">
+      <c r="E91" s="25">
         <v>4</v>
       </c>
-      <c r="F91" s="34" t="s">
+      <c r="F91" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="G91" s="33"/>
+      <c r="G91" s="25"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A92" s="18"/>
+      <c r="A92" s="28"/>
       <c r="B92" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C92" s="4">
         <v>91</v>
       </c>
-      <c r="D92" s="21" t="s">
+      <c r="D92" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="E92" s="33"/>
-      <c r="F92" s="30"/>
-      <c r="G92" s="33"/>
+      <c r="E92" s="25"/>
+      <c r="F92" s="27"/>
+      <c r="G92" s="25"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A93" s="18"/>
+      <c r="A93" s="28"/>
       <c r="B93" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C93" s="4">
         <v>92</v>
       </c>
-      <c r="D93" s="21" t="s">
+      <c r="D93" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="E93" s="33"/>
-      <c r="F93" s="30"/>
-      <c r="G93" s="33"/>
+      <c r="E93" s="25"/>
+      <c r="F93" s="27"/>
+      <c r="G93" s="25"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A94" s="18"/>
+      <c r="A94" s="28"/>
       <c r="B94" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C94" s="4">
         <v>93</v>
       </c>
-      <c r="D94" s="21" t="s">
+      <c r="D94" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="E94" s="33"/>
-      <c r="F94" s="30"/>
-      <c r="G94" s="33"/>
+      <c r="E94" s="25"/>
+      <c r="F94" s="27"/>
+      <c r="G94" s="25"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A95" s="18" t="s">
+      <c r="A95" s="28" t="s">
         <v>117</v>
       </c>
       <c r="B95" s="8" t="s">
@@ -2880,34 +2877,34 @@
       <c r="C95" s="4">
         <v>94</v>
       </c>
-      <c r="D95" s="24" t="s">
+      <c r="D95" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="E95" s="33">
+      <c r="E95" s="25">
         <v>2</v>
       </c>
-      <c r="F95" s="34" t="s">
+      <c r="F95" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="G95" s="33"/>
+      <c r="G95" s="25"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A96" s="18"/>
+      <c r="A96" s="28"/>
       <c r="B96" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C96" s="4">
         <v>95</v>
       </c>
-      <c r="D96" s="24" t="s">
+      <c r="D96" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="E96" s="33"/>
-      <c r="F96" s="30"/>
-      <c r="G96" s="33"/>
+      <c r="E96" s="25"/>
+      <c r="F96" s="27"/>
+      <c r="G96" s="25"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A97" s="18" t="s">
+      <c r="A97" s="28" t="s">
         <v>118</v>
       </c>
       <c r="B97" s="8" t="s">
@@ -2916,64 +2913,64 @@
       <c r="C97" s="4">
         <v>96</v>
       </c>
-      <c r="D97" s="21" t="s">
+      <c r="D97" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="E97" s="33">
+      <c r="E97" s="25">
         <v>4</v>
       </c>
-      <c r="F97" s="34" t="s">
+      <c r="F97" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="G97" s="33"/>
+      <c r="G97" s="25"/>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A98" s="18"/>
+      <c r="A98" s="28"/>
       <c r="B98" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C98" s="4">
         <v>97</v>
       </c>
-      <c r="D98" s="21" t="s">
+      <c r="D98" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E98" s="33"/>
-      <c r="F98" s="30"/>
-      <c r="G98" s="33"/>
+      <c r="E98" s="25"/>
+      <c r="F98" s="27"/>
+      <c r="G98" s="25"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A99" s="18"/>
+      <c r="A99" s="28"/>
       <c r="B99" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C99" s="4">
         <v>98</v>
       </c>
-      <c r="D99" s="21" t="s">
+      <c r="D99" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E99" s="33"/>
-      <c r="F99" s="30"/>
-      <c r="G99" s="33"/>
+      <c r="E99" s="25"/>
+      <c r="F99" s="27"/>
+      <c r="G99" s="25"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A100" s="18"/>
+      <c r="A100" s="28"/>
       <c r="B100" s="8" t="s">
         <v>105</v>
       </c>
       <c r="C100" s="4">
         <v>99</v>
       </c>
-      <c r="D100" s="21" t="s">
+      <c r="D100" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="E100" s="33"/>
-      <c r="F100" s="30"/>
-      <c r="G100" s="33"/>
+      <c r="E100" s="25"/>
+      <c r="F100" s="27"/>
+      <c r="G100" s="25"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A101" s="17" t="s">
+      <c r="A101" s="11" t="s">
         <v>119</v>
       </c>
       <c r="B101" s="8" t="s">
@@ -2982,16 +2979,16 @@
       <c r="C101" s="4">
         <v>100</v>
       </c>
-      <c r="D101" s="24" t="s">
+      <c r="D101" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="E101" s="32">
+      <c r="E101" s="23">
         <v>1</v>
       </c>
-      <c r="F101" s="35" t="s">
+      <c r="F101" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="G101" s="32"/>
+      <c r="G101" s="23"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A102" s="2"/>
@@ -3000,18 +2997,62 @@
     </row>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="G97:G100"/>
-    <mergeCell ref="G80:G81"/>
-    <mergeCell ref="G82:G83"/>
-    <mergeCell ref="G84:G87"/>
-    <mergeCell ref="G88:G90"/>
-    <mergeCell ref="G91:G94"/>
-    <mergeCell ref="G95:G96"/>
-    <mergeCell ref="G51:G55"/>
-    <mergeCell ref="G56:G59"/>
-    <mergeCell ref="G60:G68"/>
-    <mergeCell ref="G69:G70"/>
-    <mergeCell ref="G71:G73"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A2:A19"/>
+    <mergeCell ref="A23:A27"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A33:A38"/>
+    <mergeCell ref="A39:A43"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A44:A47"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A55"/>
+    <mergeCell ref="A56:A59"/>
+    <mergeCell ref="A88:A90"/>
+    <mergeCell ref="A91:A94"/>
+    <mergeCell ref="A95:A96"/>
+    <mergeCell ref="A97:A100"/>
+    <mergeCell ref="A60:A68"/>
+    <mergeCell ref="A80:A81"/>
+    <mergeCell ref="A82:A83"/>
+    <mergeCell ref="A84:A87"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="F2:F19"/>
+    <mergeCell ref="F20:F22"/>
+    <mergeCell ref="F23:F27"/>
+    <mergeCell ref="F28:F31"/>
+    <mergeCell ref="F33:F38"/>
+    <mergeCell ref="F39:F43"/>
+    <mergeCell ref="F44:F47"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F51:F55"/>
+    <mergeCell ref="F56:F59"/>
+    <mergeCell ref="F60:F68"/>
+    <mergeCell ref="F91:F94"/>
+    <mergeCell ref="F95:F96"/>
+    <mergeCell ref="F97:F100"/>
+    <mergeCell ref="E2:E19"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="E23:E27"/>
+    <mergeCell ref="E28:E31"/>
+    <mergeCell ref="E33:E38"/>
+    <mergeCell ref="E39:E43"/>
+    <mergeCell ref="E44:E47"/>
+    <mergeCell ref="F71:F73"/>
+    <mergeCell ref="F74:F77"/>
+    <mergeCell ref="F80:F81"/>
+    <mergeCell ref="F82:F83"/>
+    <mergeCell ref="F84:F87"/>
+    <mergeCell ref="F88:F90"/>
+    <mergeCell ref="E91:E94"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="E51:E55"/>
+    <mergeCell ref="E56:E59"/>
+    <mergeCell ref="E60:E68"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="E71:E73"/>
     <mergeCell ref="G74:G77"/>
     <mergeCell ref="E95:E96"/>
     <mergeCell ref="E97:E100"/>
@@ -3028,62 +3069,18 @@
     <mergeCell ref="E82:E83"/>
     <mergeCell ref="E84:E87"/>
     <mergeCell ref="E88:E90"/>
-    <mergeCell ref="E91:E94"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="E51:E55"/>
-    <mergeCell ref="E56:E59"/>
-    <mergeCell ref="E60:E68"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="E71:E73"/>
-    <mergeCell ref="F91:F94"/>
-    <mergeCell ref="F95:F96"/>
-    <mergeCell ref="F97:F100"/>
-    <mergeCell ref="E2:E19"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="E23:E27"/>
-    <mergeCell ref="E28:E31"/>
-    <mergeCell ref="E33:E38"/>
-    <mergeCell ref="E39:E43"/>
-    <mergeCell ref="E44:E47"/>
-    <mergeCell ref="F71:F73"/>
-    <mergeCell ref="F74:F77"/>
-    <mergeCell ref="F80:F81"/>
-    <mergeCell ref="F82:F83"/>
-    <mergeCell ref="F84:F87"/>
-    <mergeCell ref="F88:F90"/>
-    <mergeCell ref="F44:F47"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F51:F55"/>
-    <mergeCell ref="F56:F59"/>
-    <mergeCell ref="F60:F68"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="F2:F19"/>
-    <mergeCell ref="F20:F22"/>
-    <mergeCell ref="F23:F27"/>
-    <mergeCell ref="F28:F31"/>
-    <mergeCell ref="F33:F38"/>
-    <mergeCell ref="F39:F43"/>
-    <mergeCell ref="A88:A90"/>
-    <mergeCell ref="A91:A94"/>
-    <mergeCell ref="A95:A96"/>
-    <mergeCell ref="A97:A100"/>
-    <mergeCell ref="A60:A68"/>
-    <mergeCell ref="A33:A38"/>
-    <mergeCell ref="A39:A43"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A71:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A80:A81"/>
-    <mergeCell ref="A82:A83"/>
-    <mergeCell ref="A84:A87"/>
-    <mergeCell ref="A44:A47"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A55"/>
-    <mergeCell ref="A56:A59"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="A2:A19"/>
-    <mergeCell ref="A23:A27"/>
-    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="G51:G55"/>
+    <mergeCell ref="G56:G59"/>
+    <mergeCell ref="G60:G68"/>
+    <mergeCell ref="G69:G70"/>
+    <mergeCell ref="G71:G73"/>
+    <mergeCell ref="G97:G100"/>
+    <mergeCell ref="G80:G81"/>
+    <mergeCell ref="G82:G83"/>
+    <mergeCell ref="G84:G87"/>
+    <mergeCell ref="G88:G90"/>
+    <mergeCell ref="G91:G94"/>
+    <mergeCell ref="G95:G96"/>
   </mergeCells>
   <conditionalFormatting sqref="G23:G27">
     <cfRule type="dataBar" priority="1">

</xml_diff>